<commit_message>
Add watched status to Excel imports
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/film-archive-template.xlsx
+++ b/film-archive-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:Q2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,33 +410,45 @@
         <v>Row</v>
       </c>
       <c r="D1" t="str">
+        <v>Format</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Watched</v>
+      </c>
+      <c r="F1" t="str">
         <v>Director</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Cast</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Year</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Genre</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Rating</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Runtime</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Country</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
+        <v>Studio</v>
+      </c>
+      <c r="N1" t="str">
+        <v>MPA Rating</v>
+      </c>
+      <c r="O1" t="str">
         <v>Synopsis</v>
       </c>
-      <c r="L1" t="str">
+      <c r="P1" t="str">
         <v>Poster URL</v>
       </c>
-      <c r="M1" t="str">
+      <c r="Q1" t="str">
         <v>Original Title</v>
       </c>
     </row>
@@ -451,39 +463,51 @@
         <v>3</v>
       </c>
       <c r="D2" t="str">
+        <v>4K UHD</v>
+      </c>
+      <c r="E2" t="str">
+        <v>No</v>
+      </c>
+      <c r="F2" t="str">
         <v>Francis Ford Coppola</v>
       </c>
-      <c r="E2" t="str">
+      <c r="G2" t="str">
         <v>Marlon Brando, Al Pacino</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>1972</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>Crime, Drama</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>9.2</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>175</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>USA</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
+        <v>Paramount Pictures</v>
+      </c>
+      <c r="N2" t="str">
+        <v>R</v>
+      </c>
+      <c r="O2" t="str">
         <v>Story of the Corleone crime family</v>
       </c>
-      <c r="L2" t="str">
+      <c r="P2" t="str">
         <v>https://example.com/poster.jpg</v>
       </c>
-      <c r="M2" t="str">
+      <c r="Q2" t="str">
         <v>The Godfather</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>